<commit_message>
Update nodes with new version
</commit_message>
<xml_diff>
--- a/H2material.xlsx
+++ b/H2material.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\comfyUI-new\ComfyUI\custom_nodes\ComfyUI-HappNodeSet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{142CE8A9-42FC-43F9-A505-A3BD474531B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4FA0C15-C599-4CF2-ADF3-6A08FE6CA6A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{09F81F89-6F0A-48E6-9CDE-7C010105A2A2}"/>
+    <workbookView xWindow="3150" yWindow="1035" windowWidth="22740" windowHeight="14280" xr2:uid="{09F81F89-6F0A-48E6-9CDE-7C010105A2A2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>